<commit_message>
📊 [auto] Economic data update — 2026-09-25 17:43 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-09-25.xlsx
+++ b/reports/excel/MacroPulse_2026-09-25.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>3.392e+05</t>
+          <t>3.386e+05</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>-0.02%</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -24468,17 +24468,17 @@
       </c>
       <c r="N121" s="20" t="inlineStr">
         <is>
-          <t>3.357e+05</t>
+          <t>3.358e+05</t>
         </is>
       </c>
       <c r="O121" s="20" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>7.70%</t>
         </is>
       </c>
       <c r="P121" s="20" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>0.58%</t>
         </is>
       </c>
     </row>
@@ -24550,17 +24550,17 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>3.392e+05</t>
+          <t>3.387e+05</t>
         </is>
       </c>
       <c r="O122" s="19" t="inlineStr">
         <is>
-          <t>11.95%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="P122" s="19" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>0.86%</t>
         </is>
       </c>
     </row>
@@ -24632,17 +24632,17 @@
       </c>
       <c r="N123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3.386e+05</t>
         </is>
       </c>
       <c r="O123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>8.48%</t>
         </is>
       </c>
       <c r="P123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.02%</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>
@@ -59729,7 +59729,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-09-25 00:42 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-09-25 17:43 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>